<commit_message>
GGMI July: narrative revision vs canonical June deck, Renzo rulings applied (geo framing, combined KPI, funnel pending)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/forex/ggmi/2026-07/model/GGMI-July-2026-cross-channel-model.xlsx
+++ b/reports/forex/ggmi/2026-07/model/GGMI-July-2026-cross-channel-model.xlsx
@@ -595,7 +595,7 @@
         <v>4250494</v>
       </c>
       <c r="D6" t="n">
-        <v>91153</v>
+        <v>74489</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -661,7 +661,7 @@
         <v>80581160</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>137299</v>
+        <v>120635</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
@@ -699,7 +699,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Platform/vendor delivery figures. Native = Azerion native + Quantcast NativeOnly combined (tracker structure). Meta clicks = all clicks (June-consistent); link clicks 74,489 in channel workbook.</t>
+          <t>Platform/vendor delivery figures. Native = Azerion native + Quantcast NativeOnly combined (tracker structure). Meta clicks = LINK clicks per the June deck definition (June 407,136); all clicks 91,153 stay in the channel workbook.</t>
         </is>
       </c>
     </row>

</xml_diff>